<commit_message>
fix(cms): update address for SPSBP170901 to Sector 102 Suncity Avenue Gurugram
</commit_message>
<xml_diff>
--- a/CMS SITES FOR AUDITING revised.xlsx
+++ b/CMS SITES FOR AUDITING revised.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\m15250\Desktop\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{6B839C60-6D38-4D67-AB5D-A9F4DB136A51}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6F96FBF2-F094-4AB0-A1EC-8476BB6E55B6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -266,9 +266,6 @@
     <t>SECT 102 GURUGRAM</t>
   </si>
   <si>
-    <t>Shop No. 262,263 264, Plot C 01, Sector 4, Gaur City Centre, Greater Noida West</t>
-  </si>
-  <si>
     <t>SPSBV072401</t>
   </si>
   <si>
@@ -501,6 +498,9 @@
   </si>
   <si>
     <t>NIKHIL KUMAR CHATRANI</t>
+  </si>
+  <si>
+    <t>Sector 102 Suncity Avenue Gurugram</t>
   </si>
 </sst>
 </file>
@@ -629,7 +629,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="20">
+  <cellXfs count="21">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
@@ -664,6 +664,9 @@
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" wrapText="1"/>
@@ -975,8 +978,8 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:18" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A1" s="19" t="s">
-        <v>144</v>
+      <c r="A1" s="20" t="s">
+        <v>143</v>
       </c>
       <c r="B1" s="13"/>
       <c r="C1" s="13"/>
@@ -998,7 +1001,7 @@
     </row>
     <row r="2" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A2" s="6" t="s">
-        <v>145</v>
+        <v>144</v>
       </c>
       <c r="B2" s="1" t="s">
         <v>0</v>
@@ -1044,8 +1047,8 @@
       <c r="D3" s="6" t="s">
         <v>18</v>
       </c>
-      <c r="E3" s="15" t="s">
-        <v>147</v>
+      <c r="E3" s="16" t="s">
+        <v>146</v>
       </c>
       <c r="F3" s="10" t="s">
         <v>12</v>
@@ -1080,13 +1083,13 @@
       <c r="D4" s="6" t="s">
         <v>24</v>
       </c>
-      <c r="E4" s="15" t="s">
-        <v>148</v>
+      <c r="E4" s="16" t="s">
+        <v>147</v>
       </c>
       <c r="F4" s="10" t="s">
         <v>11</v>
       </c>
-      <c r="G4" s="15">
+      <c r="G4" s="16">
         <v>8860738754</v>
       </c>
       <c r="H4" s="6" t="s">
@@ -1332,13 +1335,13 @@
       <c r="D11" s="6" t="s">
         <v>57</v>
       </c>
-      <c r="E11" s="15" t="s">
-        <v>149</v>
+      <c r="E11" s="16" t="s">
+        <v>148</v>
       </c>
       <c r="F11" s="10" t="s">
         <v>12</v>
       </c>
-      <c r="G11" s="15">
+      <c r="G11" s="16">
         <v>9871287597</v>
       </c>
       <c r="H11" s="6" t="s">
@@ -1410,7 +1413,7 @@
       <c r="F13" s="10" t="s">
         <v>11</v>
       </c>
-      <c r="G13" s="15">
+      <c r="G13" s="16">
         <v>9619634856</v>
       </c>
       <c r="H13" s="6" t="s">
@@ -1462,7 +1465,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="15" spans="1:18" ht="45" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:18" ht="30" x14ac:dyDescent="0.25">
       <c r="A15" s="6">
         <f t="shared" si="0"/>
         <v>13</v>
@@ -1471,25 +1474,25 @@
         <v>74</v>
       </c>
       <c r="C15" s="6" t="s">
-        <v>150</v>
+        <v>149</v>
       </c>
       <c r="D15" s="6" t="s">
         <v>75</v>
       </c>
-      <c r="E15" s="15" t="s">
-        <v>151</v>
-      </c>
-      <c r="F15" s="15" t="s">
+      <c r="E15" s="16" t="s">
+        <v>150</v>
+      </c>
+      <c r="F15" s="16" t="s">
         <v>14</v>
       </c>
-      <c r="G15" s="15">
+      <c r="G15" s="16">
         <v>9463169925</v>
       </c>
       <c r="H15" s="6" t="s">
         <v>19</v>
       </c>
-      <c r="I15" s="8" t="s">
-        <v>76</v>
+      <c r="I15" s="15" t="s">
+        <v>154</v>
       </c>
       <c r="J15" s="12" t="s">
         <v>21</v>
@@ -1504,28 +1507,28 @@
         <v>14</v>
       </c>
       <c r="B16" s="4" t="s">
+        <v>76</v>
+      </c>
+      <c r="C16" s="6" t="s">
         <v>77</v>
       </c>
-      <c r="C16" s="6" t="s">
+      <c r="D16" s="6" t="s">
         <v>78</v>
       </c>
-      <c r="D16" s="6" t="s">
-        <v>79</v>
-      </c>
-      <c r="E16" s="15" t="s">
+      <c r="E16" s="16" t="s">
         <v>67</v>
       </c>
       <c r="F16" s="10" t="s">
         <v>14</v>
       </c>
-      <c r="G16" s="15">
+      <c r="G16" s="16">
         <v>8527194747</v>
       </c>
       <c r="H16" s="6" t="s">
         <v>19</v>
       </c>
       <c r="I16" s="8" t="s">
-        <v>80</v>
+        <v>79</v>
       </c>
       <c r="J16" s="12" t="s">
         <v>21</v>
@@ -1540,16 +1543,16 @@
         <v>15</v>
       </c>
       <c r="B17" s="4" t="s">
+        <v>80</v>
+      </c>
+      <c r="C17" s="6" t="s">
         <v>81</v>
       </c>
-      <c r="C17" s="6" t="s">
+      <c r="D17" s="6" t="s">
         <v>82</v>
       </c>
-      <c r="D17" s="6" t="s">
+      <c r="E17" s="10" t="s">
         <v>83</v>
-      </c>
-      <c r="E17" s="10" t="s">
-        <v>84</v>
       </c>
       <c r="F17" s="10" t="s">
         <v>11</v>
@@ -1561,7 +1564,7 @@
         <v>19</v>
       </c>
       <c r="I17" s="8" t="s">
-        <v>85</v>
+        <v>84</v>
       </c>
       <c r="J17" s="12" t="s">
         <v>21</v>
@@ -1576,16 +1579,16 @@
         <v>16</v>
       </c>
       <c r="B18" s="4" t="s">
+        <v>85</v>
+      </c>
+      <c r="C18" s="6" t="s">
         <v>86</v>
       </c>
-      <c r="C18" s="6" t="s">
+      <c r="D18" s="6" t="s">
         <v>87</v>
       </c>
-      <c r="D18" s="6" t="s">
+      <c r="E18" s="10" t="s">
         <v>88</v>
-      </c>
-      <c r="E18" s="10" t="s">
-        <v>89</v>
       </c>
       <c r="F18" s="10" t="s">
         <v>11</v>
@@ -1597,7 +1600,7 @@
         <v>19</v>
       </c>
       <c r="I18" s="8" t="s">
-        <v>90</v>
+        <v>89</v>
       </c>
       <c r="J18" s="12" t="s">
         <v>21</v>
@@ -1612,16 +1615,16 @@
         <v>17</v>
       </c>
       <c r="B19" s="4" t="s">
+        <v>90</v>
+      </c>
+      <c r="C19" s="6" t="s">
         <v>91</v>
       </c>
-      <c r="C19" s="6" t="s">
+      <c r="D19" s="6" t="s">
         <v>92</v>
       </c>
-      <c r="D19" s="6" t="s">
+      <c r="E19" s="10" t="s">
         <v>93</v>
-      </c>
-      <c r="E19" s="10" t="s">
-        <v>94</v>
       </c>
       <c r="F19" s="10" t="s">
         <v>14</v>
@@ -1633,7 +1636,7 @@
         <v>19</v>
       </c>
       <c r="I19" s="8" t="s">
-        <v>95</v>
+        <v>94</v>
       </c>
       <c r="J19" s="12" t="s">
         <v>21</v>
@@ -1648,28 +1651,28 @@
         <v>18</v>
       </c>
       <c r="B20" s="4" t="s">
+        <v>95</v>
+      </c>
+      <c r="C20" s="6" t="s">
         <v>96</v>
       </c>
-      <c r="C20" s="6" t="s">
+      <c r="D20" s="6" t="s">
         <v>97</v>
       </c>
-      <c r="D20" s="6" t="s">
-        <v>98</v>
-      </c>
-      <c r="E20" s="15" t="s">
-        <v>152</v>
+      <c r="E20" s="16" t="s">
+        <v>151</v>
       </c>
       <c r="F20" s="10" t="s">
         <v>11</v>
       </c>
-      <c r="G20" s="15">
+      <c r="G20" s="16">
         <v>9971976653</v>
       </c>
       <c r="H20" s="6" t="s">
         <v>19</v>
       </c>
       <c r="I20" s="8" t="s">
-        <v>99</v>
+        <v>98</v>
       </c>
       <c r="J20" s="12" t="s">
         <v>21</v>
@@ -1684,16 +1687,16 @@
         <v>19</v>
       </c>
       <c r="B21" s="4" t="s">
+        <v>99</v>
+      </c>
+      <c r="C21" s="6" t="s">
         <v>100</v>
       </c>
-      <c r="C21" s="6" t="s">
+      <c r="D21" s="6" t="s">
         <v>101</v>
       </c>
-      <c r="D21" s="6" t="s">
+      <c r="E21" s="10" t="s">
         <v>102</v>
-      </c>
-      <c r="E21" s="10" t="s">
-        <v>103</v>
       </c>
       <c r="F21" s="10" t="s">
         <v>14</v>
@@ -1705,7 +1708,7 @@
         <v>19</v>
       </c>
       <c r="I21" s="8" t="s">
-        <v>104</v>
+        <v>103</v>
       </c>
       <c r="J21" s="12" t="s">
         <v>21</v>
@@ -1720,16 +1723,16 @@
         <v>20</v>
       </c>
       <c r="B22" s="4" t="s">
+        <v>104</v>
+      </c>
+      <c r="C22" s="6" t="s">
         <v>105</v>
       </c>
-      <c r="C22" s="6" t="s">
+      <c r="D22" s="6" t="s">
         <v>106</v>
       </c>
-      <c r="D22" s="6" t="s">
+      <c r="E22" s="10" t="s">
         <v>107</v>
-      </c>
-      <c r="E22" s="10" t="s">
-        <v>108</v>
       </c>
       <c r="F22" s="10" t="s">
         <v>11</v>
@@ -1741,7 +1744,7 @@
         <v>19</v>
       </c>
       <c r="I22" s="8" t="s">
-        <v>109</v>
+        <v>108</v>
       </c>
       <c r="J22" s="12" t="s">
         <v>21</v>
@@ -1756,16 +1759,16 @@
         <v>21</v>
       </c>
       <c r="B23" s="4" t="s">
+        <v>109</v>
+      </c>
+      <c r="C23" s="6" t="s">
         <v>110</v>
       </c>
-      <c r="C23" s="6" t="s">
+      <c r="D23" s="6" t="s">
         <v>111</v>
       </c>
-      <c r="D23" s="6" t="s">
+      <c r="E23" s="10" t="s">
         <v>112</v>
-      </c>
-      <c r="E23" s="10" t="s">
-        <v>113</v>
       </c>
       <c r="F23" s="10" t="s">
         <v>11</v>
@@ -1777,7 +1780,7 @@
         <v>19</v>
       </c>
       <c r="I23" s="8" t="s">
-        <v>114</v>
+        <v>113</v>
       </c>
       <c r="J23" s="12" t="s">
         <v>21</v>
@@ -1792,16 +1795,16 @@
         <v>22</v>
       </c>
       <c r="B24" s="4" t="s">
+        <v>114</v>
+      </c>
+      <c r="C24" s="6" t="s">
         <v>115</v>
       </c>
-      <c r="C24" s="6" t="s">
+      <c r="D24" s="6" t="s">
         <v>116</v>
       </c>
-      <c r="D24" s="6" t="s">
+      <c r="E24" s="10" t="s">
         <v>117</v>
-      </c>
-      <c r="E24" s="10" t="s">
-        <v>118</v>
       </c>
       <c r="F24" s="10" t="s">
         <v>11</v>
@@ -1813,7 +1816,7 @@
         <v>19</v>
       </c>
       <c r="I24" s="8" t="s">
-        <v>119</v>
+        <v>118</v>
       </c>
       <c r="J24" s="12" t="s">
         <v>21</v>
@@ -1828,16 +1831,16 @@
         <v>23</v>
       </c>
       <c r="B25" s="4" t="s">
+        <v>119</v>
+      </c>
+      <c r="C25" s="6" t="s">
         <v>120</v>
       </c>
-      <c r="C25" s="6" t="s">
+      <c r="D25" s="6" t="s">
         <v>121</v>
       </c>
-      <c r="D25" s="6" t="s">
+      <c r="E25" s="10" t="s">
         <v>122</v>
-      </c>
-      <c r="E25" s="10" t="s">
-        <v>123</v>
       </c>
       <c r="F25" s="10" t="s">
         <v>11</v>
@@ -1849,7 +1852,7 @@
         <v>19</v>
       </c>
       <c r="I25" s="8" t="s">
-        <v>124</v>
+        <v>123</v>
       </c>
       <c r="J25" s="12" t="s">
         <v>21</v>
@@ -1864,16 +1867,16 @@
         <v>24</v>
       </c>
       <c r="B26" s="4" t="s">
+        <v>124</v>
+      </c>
+      <c r="C26" s="6" t="s">
         <v>125</v>
       </c>
-      <c r="C26" s="6" t="s">
+      <c r="D26" s="6" t="s">
         <v>126</v>
       </c>
-      <c r="D26" s="6" t="s">
+      <c r="E26" s="10" t="s">
         <v>127</v>
-      </c>
-      <c r="E26" s="10" t="s">
-        <v>128</v>
       </c>
       <c r="F26" s="10" t="s">
         <v>14</v>
@@ -1885,7 +1888,7 @@
         <v>19</v>
       </c>
       <c r="I26" s="8" t="s">
-        <v>129</v>
+        <v>128</v>
       </c>
       <c r="J26" s="12" t="s">
         <v>21</v>
@@ -1900,28 +1903,28 @@
         <v>25</v>
       </c>
       <c r="B27" s="4" t="s">
+        <v>129</v>
+      </c>
+      <c r="C27" s="6" t="s">
         <v>130</v>
       </c>
-      <c r="C27" s="6" t="s">
+      <c r="D27" s="6" t="s">
         <v>131</v>
       </c>
-      <c r="D27" s="6" t="s">
-        <v>132</v>
-      </c>
-      <c r="E27" s="15" t="s">
-        <v>153</v>
+      <c r="E27" s="16" t="s">
+        <v>152</v>
       </c>
       <c r="F27" s="10" t="s">
         <v>14</v>
       </c>
-      <c r="G27" s="15">
+      <c r="G27" s="16">
         <v>8506946777</v>
       </c>
       <c r="H27" s="6" t="s">
         <v>19</v>
       </c>
       <c r="I27" s="8" t="s">
-        <v>133</v>
+        <v>132</v>
       </c>
       <c r="J27" s="12" t="s">
         <v>21</v>
@@ -1935,17 +1938,17 @@
         <f t="shared" si="0"/>
         <v>26</v>
       </c>
-      <c r="B28" s="16" t="s">
+      <c r="B28" s="17" t="s">
+        <v>133</v>
+      </c>
+      <c r="C28" s="5" t="s">
         <v>134</v>
       </c>
-      <c r="C28" s="5" t="s">
+      <c r="D28" s="5" t="s">
         <v>135</v>
       </c>
-      <c r="D28" s="5" t="s">
-        <v>136</v>
-      </c>
       <c r="E28" s="10" t="s">
-        <v>146</v>
+        <v>145</v>
       </c>
       <c r="F28" s="10" t="s">
         <v>11</v>
@@ -1954,13 +1957,13 @@
         <v>7838424045</v>
       </c>
       <c r="H28" s="5" t="s">
+        <v>136</v>
+      </c>
+      <c r="I28" s="7" t="s">
         <v>137</v>
       </c>
-      <c r="I28" s="7" t="s">
+      <c r="J28" s="18" t="s">
         <v>138</v>
-      </c>
-      <c r="J28" s="17" t="s">
-        <v>139</v>
       </c>
       <c r="K28" s="5" t="s">
         <v>10</v>
@@ -1972,31 +1975,31 @@
         <v>27</v>
       </c>
       <c r="B29" s="4" t="s">
+        <v>139</v>
+      </c>
+      <c r="C29" s="6" t="s">
         <v>140</v>
       </c>
-      <c r="C29" s="6" t="s">
+      <c r="D29" s="6" t="s">
         <v>141</v>
       </c>
-      <c r="D29" s="6" t="s">
-        <v>142</v>
-      </c>
-      <c r="E29" s="18" t="s">
-        <v>154</v>
+      <c r="E29" s="19" t="s">
+        <v>153</v>
       </c>
       <c r="F29" s="11" t="s">
         <v>14</v>
       </c>
-      <c r="G29" s="18">
+      <c r="G29" s="19">
         <v>8963005067</v>
       </c>
       <c r="H29" s="6" t="s">
-        <v>137</v>
+        <v>136</v>
       </c>
       <c r="I29" s="8" t="s">
-        <v>143</v>
+        <v>142</v>
       </c>
       <c r="J29" s="12" t="s">
-        <v>139</v>
+        <v>138</v>
       </c>
       <c r="K29" s="6" t="s">
         <v>10</v>

</xml_diff>